<commit_message>
Add reviewed tweets REVIEWED_MorrisRamen_20161002_20191011_20260810_autoPush.xlsx
</commit_message>
<xml_diff>
--- a/reviews/REVIEWED_MorrisRamen_20161002_20191011_20260810_autoPush.xlsx
+++ b/reviews/REVIEWED_MorrisRamen_20161002_20191011_20260810_autoPush.xlsx
@@ -6289,7 +6289,7 @@
         </is>
       </c>
       <c r="H162" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I162" t="inlineStr"/>
     </row>
@@ -6320,7 +6320,7 @@
         </is>
       </c>
       <c r="H163" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I163" t="inlineStr"/>
     </row>
@@ -6358,7 +6358,7 @@
         </is>
       </c>
       <c r="H164" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I164" t="inlineStr"/>
     </row>
@@ -6393,7 +6393,7 @@
         </is>
       </c>
       <c r="H165" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I165" t="inlineStr"/>
     </row>
@@ -6429,9 +6429,13 @@
         </is>
       </c>
       <c r="H166" t="b">
-        <v>0</v>
-      </c>
-      <c r="I166" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>PLANNED PARENTHOOD</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -6464,7 +6468,7 @@
         </is>
       </c>
       <c r="H167" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I167" t="inlineStr"/>
     </row>
@@ -6502,9 +6506,13 @@
         </is>
       </c>
       <c r="H168" t="b">
-        <v>0</v>
-      </c>
-      <c r="I168" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>PERSONAL</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -6539,7 +6547,7 @@
         </is>
       </c>
       <c r="H169" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I169" t="inlineStr"/>
     </row>
@@ -6580,7 +6588,7 @@
         </is>
       </c>
       <c r="H170" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I170" t="inlineStr"/>
     </row>
@@ -6617,7 +6625,7 @@
         </is>
       </c>
       <c r="H171" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I171" t="inlineStr"/>
     </row>
@@ -6653,7 +6661,7 @@
         </is>
       </c>
       <c r="H172" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I172" t="inlineStr"/>
     </row>
@@ -6688,7 +6696,7 @@
         </is>
       </c>
       <c r="H173" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I173" t="inlineStr"/>
     </row>
@@ -6723,7 +6731,7 @@
         </is>
       </c>
       <c r="H174" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I174" t="inlineStr"/>
     </row>
@@ -6758,7 +6766,7 @@
         </is>
       </c>
       <c r="H175" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I175" t="inlineStr"/>
     </row>
@@ -6796,9 +6804,13 @@
         </is>
       </c>
       <c r="H176" t="b">
-        <v>0</v>
-      </c>
-      <c r="I176" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>PLANNED PARENTHOOD</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -6832,7 +6844,7 @@
         </is>
       </c>
       <c r="H177" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I177" t="inlineStr"/>
     </row>
@@ -6876,7 +6888,7 @@
         </is>
       </c>
       <c r="H178" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I178" t="inlineStr"/>
     </row>
@@ -6911,7 +6923,7 @@
         </is>
       </c>
       <c r="H179" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I179" t="inlineStr"/>
     </row>
@@ -6949,7 +6961,7 @@
         </is>
       </c>
       <c r="H180" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I180" t="inlineStr"/>
     </row>
@@ -6990,7 +7002,7 @@
         </is>
       </c>
       <c r="H181" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I181" t="inlineStr"/>
     </row>

</xml_diff>